<commit_message>
Added test for functionality of electrode check
Changed the nan check to an array and then printed the string representation of the string
in the warning message.

Added tests to the existing pytest for datasheet loader, now testing to make sure that
warning messages are only shown for empty cells and that the correct contacts are printed
in the warning message
</commit_message>
<xml_diff>
--- a/data/clinical_examples/electrode_layouts/test_electrode_layout.xlsx
+++ b/data/clinical_examples/electrode_layouts/test_electrode_layout.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11013"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adam2392/Documents/eegio/data/clinical_examples/electrode_layouts/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/patrick/Desktop/eegio/data/clinical_examples/electrode_layouts/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6A7B835-9C09-2343-9B2C-ABD71118EFC6}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8ACB3AD-1AB6-F24C-8426-099D29C8ADE6}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5960" yWindow="460" windowWidth="27640" windowHeight="16200" xr2:uid="{E8D599BF-346F-FF46-9897-315240A88F33}"/>
+    <workbookView xWindow="1160" yWindow="460" windowWidth="27640" windowHeight="16200" xr2:uid="{E8D599BF-346F-FF46-9897-315240A88F33}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="69">
   <si>
     <t>WM</t>
   </si>
@@ -1416,7 +1416,9 @@
       <c r="P13" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="Q13" s="13"/>
+      <c r="Q13" s="13" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="14" spans="1:17" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">

</xml_diff>